<commit_message>
Refactor: Unificación de reportes PDF bajo principio DRY y actualización de .gitignore
</commit_message>
<xml_diff>
--- a/Docs/Bloque Asignaciones Detalles.xlsx
+++ b/Docs/Bloque Asignaciones Detalles.xlsx
@@ -8,16 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Desarrollos\MyPython\Tkinter\ArkConInv\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6284DB43-13C8-4568-890B-F66627EF132B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F4DDAEBD-5F91-4D83-8043-0466AE3CDEE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="766" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bloque Asignaciones SDetalleVta" sheetId="1" r:id="rId1"/>
     <sheet name="Bloque Asignaciones SDetalleCom" sheetId="3" r:id="rId2"/>
+    <sheet name="Bloque Asignaciones DetallesInv" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -26,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="390">
   <si>
     <t>FDI_TIPOOPERACION</t>
   </si>
@@ -899,6 +909,303 @@
   </si>
   <si>
     <t>dtc_existedetalleimportacion</t>
+  </si>
+  <si>
+    <t>dtc_idunico</t>
+  </si>
+  <si>
+    <t>generar_idunico</t>
+  </si>
+  <si>
+    <t>ark_detalletrancomp</t>
+  </si>
+  <si>
+    <t>ark_detalletraninv</t>
+  </si>
+  <si>
+    <t>SDetalleInv</t>
+  </si>
+  <si>
+    <t>dti_Idauto</t>
+  </si>
+  <si>
+    <t>dti_idunico</t>
+  </si>
+  <si>
+    <t>dti_uo_id</t>
+  </si>
+  <si>
+    <t>dti_uo_Codigo</t>
+  </si>
+  <si>
+    <t>dti_tipooperacion</t>
+  </si>
+  <si>
+    <t>dti_codigo</t>
+  </si>
+  <si>
+    <t>dti_linea</t>
+  </si>
+  <si>
+    <t>dti_documento</t>
+  </si>
+  <si>
+    <t>dti_autoincrement</t>
+  </si>
+  <si>
+    <t>dti_clienteproveedor</t>
+  </si>
+  <si>
+    <t>dti_tipodocumentoorigen</t>
+  </si>
+  <si>
+    <t>dti_statusdocumentoorigen</t>
+  </si>
+  <si>
+    <t>dti_documentoorigen</t>
+  </si>
+  <si>
+    <t>dti_lineaorigen</t>
+  </si>
+  <si>
+    <t>dti_clasificacion</t>
+  </si>
+  <si>
+    <t>dti_status</t>
+  </si>
+  <si>
+    <t>dti_visible</t>
+  </si>
+  <si>
+    <t>dti_costo</t>
+  </si>
+  <si>
+    <t>dti_cantidad</t>
+  </si>
+  <si>
+    <t>dti_cantidadpendiente</t>
+  </si>
+  <si>
+    <t>dti_lote</t>
+  </si>
+  <si>
+    <t>dti_loterandom</t>
+  </si>
+  <si>
+    <t>dti_newlote</t>
+  </si>
+  <si>
+    <t>dti_depositosource</t>
+  </si>
+  <si>
+    <t>dti_depositotarget</t>
+  </si>
+  <si>
+    <t>dti_operacion_autoincrement</t>
+  </si>
+  <si>
+    <t>dti_decimales</t>
+  </si>
+  <si>
+    <t>dti_decimalespen</t>
+  </si>
+  <si>
+    <t>dti_serialnumber</t>
+  </si>
+  <si>
+    <t>dti_usaseriales</t>
+  </si>
+  <si>
+    <t>dti_usadepositos</t>
+  </si>
+  <si>
+    <t>dti_costooperacion</t>
+  </si>
+  <si>
+    <t>dti_memodetalle</t>
+  </si>
+  <si>
+    <t>dti_moneda</t>
+  </si>
+  <si>
+    <t>dti_factorcambio</t>
+  </si>
+  <si>
+    <t>dti_detallecostosimportacion</t>
+  </si>
+  <si>
+    <t>dti_detalleplanillaimportacion</t>
+  </si>
+  <si>
+    <t>dti_existedetalleimportacion</t>
+  </si>
+  <si>
+    <t>dti_existedetalledecostos</t>
+  </si>
+  <si>
+    <t>dti_alicuotafleteotros</t>
+  </si>
+  <si>
+    <t>dti_impuesto1</t>
+  </si>
+  <si>
+    <t>dti_porcentimpuesto1</t>
+  </si>
+  <si>
+    <t>dti_montoimpuesto1</t>
+  </si>
+  <si>
+    <t>dti_impuesto2</t>
+  </si>
+  <si>
+    <t>dti_porcentimpuesto2</t>
+  </si>
+  <si>
+    <t>dti_montoimpuesto2</t>
+  </si>
+  <si>
+    <t>dti_origenprice</t>
+  </si>
+  <si>
+    <t>dti_porcentdescparcial</t>
+  </si>
+  <si>
+    <t>dti_descuentoparcial</t>
+  </si>
+  <si>
+    <t>dti_preciosindescuento</t>
+  </si>
+  <si>
+    <t>dti_preciocondescuento</t>
+  </si>
+  <si>
+    <t>dti_preciodeventa</t>
+  </si>
+  <si>
+    <t>dti_rounddesctparcial</t>
+  </si>
+  <si>
+    <t>dti_comisionfija</t>
+  </si>
+  <si>
+    <t>dti_comisionfijap</t>
+  </si>
+  <si>
+    <t>dti_unddescarga</t>
+  </si>
+  <si>
+    <t>dti_undcapacidad</t>
+  </si>
+  <si>
+    <t>dti_unddetallada</t>
+  </si>
+  <si>
+    <t>dti_indexprices</t>
+  </si>
+  <si>
+    <t>dti_partesusanseriales</t>
+  </si>
+  <si>
+    <t>dti_costodeventas</t>
+  </si>
+  <si>
+    <t>dti_descripcionoferta</t>
+  </si>
+  <si>
+    <t>dti_vendedorasignado</t>
+  </si>
+  <si>
+    <t>dti_montocomision</t>
+  </si>
+  <si>
+    <t>dti_preciobasecomision</t>
+  </si>
+  <si>
+    <t>dti_comisionbloqueada</t>
+  </si>
+  <si>
+    <t>dti_comisionyapagada</t>
+  </si>
+  <si>
+    <t>dti_documentoliberacion</t>
+  </si>
+  <si>
+    <t>dti_tipodecomision</t>
+  </si>
+  <si>
+    <t>dti_priceforcomision</t>
+  </si>
+  <si>
+    <t>dti_fechaoperacion</t>
+  </si>
+  <si>
+    <t>dti_user</t>
+  </si>
+  <si>
+    <t>dti_porcentdescuento1</t>
+  </si>
+  <si>
+    <t>dti_porcentdescuento2</t>
+  </si>
+  <si>
+    <t>dti_costosupdate</t>
+  </si>
+  <si>
+    <t>dti_base_autoincrement</t>
+  </si>
+  <si>
+    <t>dti_totalpeso</t>
+  </si>
+  <si>
+    <t>dti_ctocosto</t>
+  </si>
+  <si>
+    <t>dti_autorizado</t>
+  </si>
+  <si>
+    <t>dti_markperiodo</t>
+  </si>
+  <si>
+    <t>dti_ctocostostr</t>
+  </si>
+  <si>
+    <t>dti_costoactualnacional</t>
+  </si>
+  <si>
+    <t>dti_costoactualext</t>
+  </si>
+  <si>
+    <t>dti_prefixinventario</t>
+  </si>
+  <si>
+    <t>dti_costoajustado</t>
+  </si>
+  <si>
+    <t>dti_fechalibro</t>
+  </si>
+  <si>
+    <t>dti_SystemDate</t>
+  </si>
+  <si>
+    <t>dti_SystemTime</t>
+  </si>
+  <si>
+    <t>dti_NameMachine</t>
+  </si>
+  <si>
+    <t>dti_UserCreator</t>
+  </si>
+  <si>
+    <t>dti_LastUpdateDate</t>
+  </si>
+  <si>
+    <t>dti_LastUpdateTime</t>
+  </si>
+  <si>
+    <t>dti_LastMachine</t>
+  </si>
+  <si>
+    <t>dti_UserLastUpdate</t>
   </si>
 </sst>
 </file>
@@ -3464,7 +3771,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4916DF45-9F63-420F-94C1-459091540526}">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32.7109375" customWidth="1"/>
@@ -3477,7 +3784,7 @@
         <v>193</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>182</v>
+        <v>293</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>193</v>
@@ -3494,7 +3801,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>198</v>
@@ -3511,16 +3818,17 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>2</v>
+        <f>A2+1</f>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>291</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E3" t="s">
-        <v>185</v>
+        <v>292</v>
       </c>
       <c r="F3" t="s">
         <v>196</v>
@@ -3528,16 +3836,17 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>3</v>
+        <f t="shared" ref="A4:A67" si="0">A3+1</f>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F4" t="s">
         <v>196</v>
@@ -3545,16 +3854,17 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
-        <v>4</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>201</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>0</v>
+        <v>200</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" t="s">
+        <v>186</v>
       </c>
       <c r="F5" t="s">
         <v>196</v>
@@ -3562,16 +3872,17 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C6" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="s">
         <v>196</v>
@@ -3579,16 +3890,18 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <v>6</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C7" s="2">
-        <v>3</v>
+        <f>+C6+1</f>
+        <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
         <v>196</v>
@@ -3596,16 +3909,18 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>7</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C8" s="2">
-        <v>4</v>
+        <f t="shared" ref="C8:C71" si="1">+C7+1</f>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="s">
         <v>196</v>
@@ -3613,16 +3928,18 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
-        <v>8</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C9" s="2">
-        <v>5</v>
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="s">
         <v>196</v>
@@ -3630,16 +3947,18 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
-        <v>9</v>
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C10" s="2">
-        <v>6</v>
+        <f t="shared" si="1"/>
+        <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="s">
         <v>196</v>
@@ -3647,16 +3966,18 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C11" s="2">
-        <v>7</v>
+        <f t="shared" si="1"/>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>5</v>
       </c>
       <c r="F11" t="s">
         <v>196</v>
@@ -3664,16 +3985,18 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
-        <v>11</v>
+        <f t="shared" si="0"/>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C12" s="2">
-        <v>8</v>
+        <f t="shared" si="1"/>
+        <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F12" t="s">
         <v>196</v>
@@ -3681,16 +4004,18 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
-        <v>12</v>
+        <f t="shared" si="0"/>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C13" s="2">
-        <v>9</v>
+        <f t="shared" si="1"/>
+        <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
         <v>196</v>
@@ -3698,16 +4023,18 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
-        <v>13</v>
+        <f t="shared" si="0"/>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C14" s="2">
-        <v>10</v>
+        <f t="shared" si="1"/>
+        <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" t="s">
         <v>196</v>
@@ -3715,16 +4042,18 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
-        <v>14</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C15" s="2">
-        <v>11</v>
+        <f t="shared" si="1"/>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="s">
         <v>196</v>
@@ -3732,16 +4061,18 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C16" s="2">
-        <v>12</v>
+        <f t="shared" si="1"/>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" t="s">
         <v>196</v>
@@ -3749,16 +4080,18 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
-        <v>16</v>
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C17" s="2">
-        <v>13</v>
+        <f t="shared" si="1"/>
+        <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="s">
         <v>196</v>
@@ -3766,16 +4099,18 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
-        <v>17</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C18" s="2">
-        <v>14</v>
+        <f t="shared" si="1"/>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
         <v>196</v>
@@ -3783,16 +4118,18 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
-        <v>18</v>
+        <f t="shared" si="0"/>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C19" s="2">
-        <v>15</v>
+        <f t="shared" si="1"/>
+        <v>13</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F19" t="s">
         <v>196</v>
@@ -3800,16 +4137,18 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
-        <v>19</v>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C20" s="2">
-        <v>16</v>
+        <f t="shared" si="1"/>
+        <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F20" t="s">
         <v>196</v>
@@ -3817,16 +4156,18 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
-        <v>20</v>
+        <f t="shared" si="0"/>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2">
-        <v>17</v>
+        <f t="shared" si="1"/>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F21" t="s">
         <v>196</v>
@@ -3834,16 +4175,18 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
-        <v>21</v>
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C22" s="2">
-        <v>18</v>
+        <f t="shared" si="1"/>
+        <v>16</v>
       </c>
       <c r="D22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F22" t="s">
         <v>196</v>
@@ -3851,16 +4194,18 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
-        <v>22</v>
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C23" s="2">
-        <v>19</v>
+        <f t="shared" si="1"/>
+        <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F23" t="s">
         <v>196</v>
@@ -3868,16 +4213,18 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
-        <v>23</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C24" s="2">
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F24" t="s">
         <v>196</v>
@@ -3885,16 +4232,18 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
-        <v>24</v>
+        <f t="shared" si="0"/>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C25" s="2">
-        <v>21</v>
+        <f t="shared" si="1"/>
+        <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F25" t="s">
         <v>196</v>
@@ -3902,16 +4251,18 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
-        <v>25</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C26" s="2">
-        <v>22</v>
+        <f t="shared" si="1"/>
+        <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F26" t="s">
         <v>196</v>
@@ -3919,16 +4270,18 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
-        <v>26</v>
+        <f t="shared" si="0"/>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C27" s="2">
-        <v>23</v>
+        <f t="shared" si="1"/>
+        <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
         <v>196</v>
@@ -3936,16 +4289,18 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
-        <v>27</v>
+        <f t="shared" si="0"/>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C28" s="2">
-        <v>24</v>
+        <f t="shared" si="1"/>
+        <v>22</v>
       </c>
       <c r="D28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F28" t="s">
         <v>196</v>
@@ -3953,16 +4308,18 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
-        <v>28</v>
+        <f t="shared" si="0"/>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C29" s="2">
-        <v>25</v>
+        <f t="shared" si="1"/>
+        <v>23</v>
       </c>
       <c r="D29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F29" t="s">
         <v>196</v>
@@ -3970,16 +4327,18 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
-        <v>29</v>
+        <f t="shared" si="0"/>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C30" s="2">
-        <v>26</v>
+        <f t="shared" si="1"/>
+        <v>24</v>
       </c>
       <c r="D30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F30" t="s">
         <v>196</v>
@@ -3987,16 +4346,18 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
-        <v>30</v>
+        <f t="shared" si="0"/>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C31" s="2">
-        <v>27</v>
+        <f t="shared" si="1"/>
+        <v>25</v>
       </c>
       <c r="D31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F31" t="s">
         <v>196</v>
@@ -4004,16 +4365,18 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>31</v>
+        <f t="shared" si="0"/>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C32" s="2">
-        <v>28</v>
+        <f t="shared" si="1"/>
+        <v>26</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
         <v>196</v>
@@ -4021,16 +4384,18 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
-        <v>32</v>
+        <f t="shared" si="0"/>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C33" s="2">
-        <v>29</v>
+        <f t="shared" si="1"/>
+        <v>27</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F33" t="s">
         <v>196</v>
@@ -4038,16 +4403,18 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
-        <v>33</v>
+        <f t="shared" si="0"/>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C34" s="2">
-        <v>30</v>
+        <f t="shared" si="1"/>
+        <v>28</v>
       </c>
       <c r="D34" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F34" t="s">
         <v>196</v>
@@ -4055,16 +4422,18 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
-        <v>34</v>
+        <f t="shared" si="0"/>
+        <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C35" s="2">
-        <v>31</v>
+        <f t="shared" si="1"/>
+        <v>29</v>
       </c>
       <c r="D35" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F35" t="s">
         <v>196</v>
@@ -4072,16 +4441,18 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
-        <v>35</v>
+        <f t="shared" si="0"/>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>288</v>
+        <v>231</v>
       </c>
       <c r="C36" s="2">
-        <v>32</v>
+        <f t="shared" si="1"/>
+        <v>30</v>
       </c>
       <c r="D36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F36" t="s">
         <v>196</v>
@@ -4089,16 +4460,18 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
-        <v>36</v>
+        <f t="shared" si="0"/>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C37" s="2">
-        <v>33</v>
+        <f t="shared" si="1"/>
+        <v>31</v>
       </c>
       <c r="D37" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F37" t="s">
         <v>196</v>
@@ -4106,16 +4479,18 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
-        <v>37</v>
+        <f t="shared" si="0"/>
+        <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C38" s="2">
-        <v>34</v>
+        <f t="shared" si="1"/>
+        <v>32</v>
       </c>
       <c r="D38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F38" t="s">
         <v>196</v>
@@ -4123,16 +4498,18 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
-        <v>38</v>
+        <f t="shared" si="0"/>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>232</v>
+        <v>290</v>
       </c>
       <c r="C39" s="2">
-        <v>35</v>
+        <f t="shared" si="1"/>
+        <v>33</v>
       </c>
       <c r="D39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F39" t="s">
         <v>196</v>
@@ -4140,16 +4517,18 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
-        <v>39</v>
+        <f t="shared" si="0"/>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C40" s="2">
-        <v>36</v>
+        <f t="shared" si="1"/>
+        <v>34</v>
       </c>
       <c r="D40" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F40" t="s">
         <v>196</v>
@@ -4157,16 +4536,18 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
-        <v>40</v>
+        <f t="shared" si="0"/>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C41" s="2">
-        <v>37</v>
+        <f t="shared" si="1"/>
+        <v>35</v>
       </c>
       <c r="D41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F41" t="s">
         <v>196</v>
@@ -4174,16 +4555,18 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
-        <v>41</v>
+        <f t="shared" si="0"/>
+        <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C42" s="2">
-        <v>38</v>
+        <f t="shared" si="1"/>
+        <v>36</v>
       </c>
       <c r="D42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F42" t="s">
         <v>196</v>
@@ -4191,16 +4574,18 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
-        <v>42</v>
+        <f t="shared" si="0"/>
+        <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C43" s="2">
-        <v>39</v>
+        <f t="shared" si="1"/>
+        <v>37</v>
       </c>
       <c r="D43" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F43" t="s">
         <v>196</v>
@@ -4208,16 +4593,18 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
-        <v>43</v>
+        <f t="shared" si="0"/>
+        <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C44" s="2">
-        <v>40</v>
+        <f t="shared" si="1"/>
+        <v>38</v>
       </c>
       <c r="D44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F44" t="s">
         <v>196</v>
@@ -4225,16 +4612,18 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
-        <v>44</v>
+        <f t="shared" si="0"/>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C45" s="2">
-        <v>41</v>
+        <f t="shared" si="1"/>
+        <v>39</v>
       </c>
       <c r="D45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F45" t="s">
         <v>196</v>
@@ -4242,16 +4631,18 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
-        <v>45</v>
+        <f t="shared" si="0"/>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C46" s="2">
-        <v>42</v>
+        <f t="shared" si="1"/>
+        <v>40</v>
       </c>
       <c r="D46" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F46" t="s">
         <v>196</v>
@@ -4259,16 +4650,18 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
-        <v>46</v>
+        <f t="shared" si="0"/>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C47" s="2">
-        <v>43</v>
+        <f t="shared" si="1"/>
+        <v>41</v>
       </c>
       <c r="D47" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F47" t="s">
         <v>196</v>
@@ -4276,16 +4669,18 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
-        <v>47</v>
+        <f t="shared" si="0"/>
+        <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C48" s="2">
-        <v>44</v>
+        <f t="shared" si="1"/>
+        <v>42</v>
       </c>
       <c r="D48" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F48" t="s">
         <v>196</v>
@@ -4293,16 +4688,18 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
-        <v>48</v>
+        <f t="shared" si="0"/>
+        <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C49" s="2">
-        <v>45</v>
+        <f t="shared" si="1"/>
+        <v>43</v>
       </c>
       <c r="D49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F49" t="s">
         <v>196</v>
@@ -4310,16 +4707,18 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
-        <v>49</v>
+        <f t="shared" si="0"/>
+        <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C50" s="2">
-        <v>46</v>
+        <f t="shared" si="1"/>
+        <v>44</v>
       </c>
       <c r="D50" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" t="s">
         <v>196</v>
@@ -4327,16 +4726,18 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
-        <v>50</v>
+        <f t="shared" si="0"/>
+        <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C51" s="2">
-        <v>47</v>
+        <f t="shared" si="1"/>
+        <v>45</v>
       </c>
       <c r="D51" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F51" t="s">
         <v>196</v>
@@ -4344,16 +4745,18 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
-        <v>51</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C52" s="2">
-        <v>48</v>
+        <f t="shared" si="1"/>
+        <v>46</v>
       </c>
       <c r="D52" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F52" t="s">
         <v>196</v>
@@ -4361,16 +4764,18 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
-        <v>52</v>
+        <f t="shared" si="0"/>
+        <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C53" s="2">
-        <v>49</v>
+        <f t="shared" si="1"/>
+        <v>47</v>
       </c>
       <c r="D53" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F53" t="s">
         <v>196</v>
@@ -4378,16 +4783,18 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
-        <v>53</v>
+        <f t="shared" si="0"/>
+        <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C54" s="2">
-        <v>50</v>
+        <f t="shared" si="1"/>
+        <v>48</v>
       </c>
       <c r="D54" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F54" t="s">
         <v>196</v>
@@ -4395,16 +4802,18 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C55" s="2">
-        <v>51</v>
+        <f t="shared" si="1"/>
+        <v>49</v>
       </c>
       <c r="D55" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F55" t="s">
         <v>196</v>
@@ -4412,16 +4821,18 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
-        <v>55</v>
+        <f t="shared" si="0"/>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C56" s="2">
-        <v>52</v>
+        <f t="shared" si="1"/>
+        <v>50</v>
       </c>
       <c r="D56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F56" t="s">
         <v>196</v>
@@ -4429,16 +4840,18 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
-        <v>56</v>
+        <f t="shared" si="0"/>
+        <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C57" s="2">
-        <v>53</v>
+        <f t="shared" si="1"/>
+        <v>51</v>
       </c>
       <c r="D57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F57" t="s">
         <v>196</v>
@@ -4446,16 +4859,18 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
-        <v>57</v>
+        <f t="shared" si="0"/>
+        <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C58" s="2">
-        <v>54</v>
+        <f t="shared" si="1"/>
+        <v>52</v>
       </c>
       <c r="D58" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F58" t="s">
         <v>196</v>
@@ -4463,16 +4878,18 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
-        <v>58</v>
+        <f t="shared" si="0"/>
+        <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C59" s="2">
-        <v>55</v>
+        <f t="shared" si="1"/>
+        <v>53</v>
       </c>
       <c r="D59" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F59" t="s">
         <v>196</v>
@@ -4480,16 +4897,18 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
-        <v>59</v>
+        <f t="shared" si="0"/>
+        <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C60" s="2">
-        <v>56</v>
+        <f t="shared" si="1"/>
+        <v>54</v>
       </c>
       <c r="D60" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F60" t="s">
         <v>196</v>
@@ -4497,16 +4916,18 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
-        <v>60</v>
+        <f t="shared" si="0"/>
+        <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C61" s="2">
-        <v>57</v>
+        <f t="shared" si="1"/>
+        <v>55</v>
       </c>
       <c r="D61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F61" t="s">
         <v>196</v>
@@ -4514,16 +4935,18 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
-        <v>61</v>
+        <f t="shared" si="0"/>
+        <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C62" s="2">
-        <v>58</v>
+        <f t="shared" si="1"/>
+        <v>56</v>
       </c>
       <c r="D62" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F62" t="s">
         <v>196</v>
@@ -4531,16 +4954,18 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
-        <v>62</v>
+        <f t="shared" si="0"/>
+        <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C63" s="2">
-        <v>59</v>
+        <f t="shared" si="1"/>
+        <v>57</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F63" t="s">
         <v>196</v>
@@ -4548,16 +4973,18 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
-        <v>63</v>
+        <f t="shared" si="0"/>
+        <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C64" s="2">
-        <v>60</v>
+        <f t="shared" si="1"/>
+        <v>58</v>
       </c>
       <c r="D64" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F64" t="s">
         <v>196</v>
@@ -4565,16 +4992,18 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
-        <v>64</v>
+        <f t="shared" si="0"/>
+        <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C65" s="2">
-        <v>61</v>
+        <f t="shared" si="1"/>
+        <v>59</v>
       </c>
       <c r="D65" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F65" t="s">
         <v>196</v>
@@ -4582,16 +5011,18 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
-        <v>65</v>
+        <f t="shared" si="0"/>
+        <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C66" s="2">
-        <v>62</v>
+        <f t="shared" si="1"/>
+        <v>60</v>
       </c>
       <c r="D66" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F66" t="s">
         <v>196</v>
@@ -4599,16 +5030,18 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
-        <v>66</v>
+        <f t="shared" si="0"/>
+        <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C67" s="2">
-        <v>63</v>
+        <f t="shared" si="1"/>
+        <v>61</v>
       </c>
       <c r="D67" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F67" t="s">
         <v>196</v>
@@ -4616,16 +5049,18 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
-        <v>67</v>
+        <f t="shared" ref="A68:A95" si="2">A67+1</f>
+        <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C68" s="2">
-        <v>64</v>
+        <f t="shared" si="1"/>
+        <v>62</v>
       </c>
       <c r="D68" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F68" t="s">
         <v>196</v>
@@ -4633,16 +5068,18 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
-        <v>68</v>
+        <f t="shared" si="2"/>
+        <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C69" s="2">
-        <v>65</v>
+        <f t="shared" si="1"/>
+        <v>63</v>
       </c>
       <c r="D69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F69" t="s">
         <v>196</v>
@@ -4650,16 +5087,18 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
-        <v>69</v>
+        <f t="shared" si="2"/>
+        <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C70" s="2">
-        <v>66</v>
+        <f t="shared" si="1"/>
+        <v>64</v>
       </c>
       <c r="D70" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F70" t="s">
         <v>196</v>
@@ -4667,16 +5106,18 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
-        <v>70</v>
+        <f t="shared" si="2"/>
+        <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C71" s="2">
-        <v>67</v>
+        <f t="shared" si="1"/>
+        <v>65</v>
       </c>
       <c r="D71" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F71" t="s">
         <v>196</v>
@@ -4684,16 +5125,18 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
-        <v>71</v>
+        <f t="shared" si="2"/>
+        <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C72" s="2">
-        <v>68</v>
+        <f t="shared" ref="C72:C87" si="3">+C71+1</f>
+        <v>66</v>
       </c>
       <c r="D72" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F72" t="s">
         <v>196</v>
@@ -4701,16 +5144,18 @@
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
-        <v>72</v>
+        <f t="shared" si="2"/>
+        <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C73" s="2">
-        <v>69</v>
+        <f t="shared" si="3"/>
+        <v>67</v>
       </c>
       <c r="D73" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F73" t="s">
         <v>196</v>
@@ -4718,16 +5163,18 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
-        <v>73</v>
+        <f t="shared" si="2"/>
+        <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C74" s="2">
-        <v>70</v>
+        <f t="shared" si="3"/>
+        <v>68</v>
       </c>
       <c r="D74" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F74" t="s">
         <v>196</v>
@@ -4735,16 +5182,18 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
-        <v>74</v>
+        <f t="shared" si="2"/>
+        <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C75" s="2">
-        <v>71</v>
+        <f t="shared" si="3"/>
+        <v>69</v>
       </c>
       <c r="D75" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F75" t="s">
         <v>196</v>
@@ -4752,16 +5201,18 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
-        <v>75</v>
+        <f t="shared" si="2"/>
+        <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C76" s="2">
-        <v>72</v>
+        <f t="shared" si="3"/>
+        <v>70</v>
       </c>
       <c r="D76" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F76" t="s">
         <v>196</v>
@@ -4769,16 +5220,18 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
-        <v>76</v>
+        <f t="shared" si="2"/>
+        <v>75</v>
       </c>
       <c r="B77" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C77" s="2">
-        <v>73</v>
+        <f t="shared" si="3"/>
+        <v>71</v>
       </c>
       <c r="D77" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F77" t="s">
         <v>196</v>
@@ -4786,16 +5239,18 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
-        <v>77</v>
+        <f t="shared" si="2"/>
+        <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C78" s="2">
-        <v>74</v>
+        <f t="shared" si="3"/>
+        <v>72</v>
       </c>
       <c r="D78" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F78" t="s">
         <v>196</v>
@@ -4803,16 +5258,18 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
-        <v>78</v>
+        <f t="shared" si="2"/>
+        <v>77</v>
       </c>
       <c r="B79" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C79" s="2">
-        <v>75</v>
+        <f t="shared" si="3"/>
+        <v>73</v>
       </c>
       <c r="D79" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F79" t="s">
         <v>196</v>
@@ -4820,16 +5277,18 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
-        <v>79</v>
+        <f t="shared" si="2"/>
+        <v>78</v>
       </c>
       <c r="B80" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C80" s="2">
-        <v>76</v>
+        <f t="shared" si="3"/>
+        <v>74</v>
       </c>
       <c r="D80" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F80" t="s">
         <v>196</v>
@@ -4837,16 +5296,18 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
-        <v>80</v>
+        <f t="shared" si="2"/>
+        <v>79</v>
       </c>
       <c r="B81" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C81" s="2">
-        <v>77</v>
+        <f t="shared" si="3"/>
+        <v>75</v>
       </c>
       <c r="D81" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F81" t="s">
         <v>196</v>
@@ -4854,16 +5315,18 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
-        <v>81</v>
+        <f t="shared" si="2"/>
+        <v>80</v>
       </c>
       <c r="B82" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C82" s="2">
-        <v>78</v>
+        <f t="shared" si="3"/>
+        <v>76</v>
       </c>
       <c r="D82" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F82" t="s">
         <v>196</v>
@@ -4871,16 +5334,18 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
-        <v>82</v>
+        <f t="shared" si="2"/>
+        <v>81</v>
       </c>
       <c r="B83" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C83" s="2">
-        <v>79</v>
+        <f t="shared" si="3"/>
+        <v>77</v>
       </c>
       <c r="D83" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F83" t="s">
         <v>196</v>
@@ -4888,16 +5353,18 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
-        <v>83</v>
+        <f t="shared" si="2"/>
+        <v>82</v>
       </c>
       <c r="B84" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C84" s="2">
-        <v>80</v>
+        <f t="shared" si="3"/>
+        <v>78</v>
       </c>
       <c r="D84" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F84" t="s">
         <v>196</v>
@@ -4905,16 +5372,18 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
-        <v>84</v>
+        <f t="shared" si="2"/>
+        <v>83</v>
       </c>
       <c r="B85" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C85" s="2">
-        <v>81</v>
+        <f t="shared" si="3"/>
+        <v>79</v>
       </c>
       <c r="D85" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F85" t="s">
         <v>196</v>
@@ -4922,16 +5391,18 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
-        <v>85</v>
+        <f t="shared" si="2"/>
+        <v>84</v>
       </c>
       <c r="B86" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C86" s="2">
-        <v>82</v>
+        <f t="shared" si="3"/>
+        <v>80</v>
       </c>
       <c r="D86" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F86" t="s">
         <v>196</v>
@@ -4939,16 +5410,18 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
-        <v>86</v>
+        <f t="shared" si="2"/>
+        <v>85</v>
       </c>
       <c r="B87" t="s">
-        <v>280</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E87" t="s">
-        <v>189</v>
+        <v>279</v>
+      </c>
+      <c r="C87" s="2">
+        <f t="shared" si="3"/>
+        <v>81</v>
+      </c>
+      <c r="D87" t="s">
+        <v>79</v>
       </c>
       <c r="F87" t="s">
         <v>196</v>
@@ -4956,16 +5429,17 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
-        <v>87</v>
+        <f t="shared" si="2"/>
+        <v>86</v>
       </c>
       <c r="B88" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E88" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F88" t="s">
         <v>196</v>
@@ -4973,16 +5447,17 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
-        <v>88</v>
+        <f t="shared" si="2"/>
+        <v>87</v>
       </c>
       <c r="B89" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E89" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="F89" t="s">
         <v>196</v>
@@ -4990,16 +5465,17 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
-        <v>89</v>
+        <f t="shared" si="2"/>
+        <v>88</v>
       </c>
       <c r="B90" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E90" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="F90" t="s">
         <v>196</v>
@@ -5007,16 +5483,17 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
-        <v>90</v>
+        <f t="shared" si="2"/>
+        <v>89</v>
       </c>
       <c r="B91" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E91" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F91" t="s">
         <v>196</v>
@@ -5024,16 +5501,17 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
-        <v>91</v>
+        <f t="shared" si="2"/>
+        <v>90</v>
       </c>
       <c r="B92" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E92" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F92" t="s">
         <v>196</v>
@@ -5041,16 +5519,17 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
-        <v>92</v>
+        <f t="shared" si="2"/>
+        <v>91</v>
       </c>
       <c r="B93" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E93" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="F93" t="s">
         <v>196</v>
@@ -5058,18 +5537,1845 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
-        <v>93</v>
+        <f t="shared" si="2"/>
+        <v>92</v>
       </c>
       <c r="B94" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>197</v>
       </c>
       <c r="E94" t="s">
+        <v>187</v>
+      </c>
+      <c r="F94" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="2">
+        <f t="shared" si="2"/>
+        <v>93</v>
+      </c>
+      <c r="B95" t="s">
+        <v>287</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E95" t="s">
         <v>190</v>
       </c>
+      <c r="F95" t="s">
+        <v>194</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A525AD9F-D77F-4B0E-AA52-CD509B1553B7}">
+  <dimension ref="A1:F95"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.85546875" customWidth="1"/>
+    <col min="5" max="5" width="36.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <f>A2+1</f>
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E3" t="s">
+        <v>292</v>
+      </c>
+      <c r="F3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <f t="shared" ref="A4:A67" si="0">A3+1</f>
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>298</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F4" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>299</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" t="s">
+        <v>186</v>
+      </c>
+      <c r="F5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>301</v>
+      </c>
+      <c r="C7" s="2">
+        <f>+C6+1</f>
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>302</v>
+      </c>
+      <c r="C8" s="2">
+        <f t="shared" ref="C8:C71" si="1">+C7+1</f>
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="2">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>304</v>
+      </c>
+      <c r="C10" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>305</v>
+      </c>
+      <c r="C11" s="2">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>306</v>
+      </c>
+      <c r="C12" s="2">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>307</v>
+      </c>
+      <c r="C13" s="2">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>308</v>
+      </c>
+      <c r="C14" s="2">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>309</v>
+      </c>
+      <c r="C15" s="2">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>310</v>
+      </c>
+      <c r="C16" s="2">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>311</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>312</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>313</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>314</v>
+      </c>
+      <c r="C20" s="2">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>315</v>
+      </c>
+      <c r="C21" s="2">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>316</v>
+      </c>
+      <c r="C22" s="2">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>317</v>
+      </c>
+      <c r="C23" s="2">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="D23" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>318</v>
+      </c>
+      <c r="C24" s="2">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>319</v>
+      </c>
+      <c r="C25" s="2">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C26" s="2">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="D26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>321</v>
+      </c>
+      <c r="C27" s="2">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="D27" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>322</v>
+      </c>
+      <c r="C28" s="2">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>323</v>
+      </c>
+      <c r="C29" s="2">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>324</v>
+      </c>
+      <c r="C30" s="2">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="D30" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>325</v>
+      </c>
+      <c r="C31" s="2">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="D31" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>326</v>
+      </c>
+      <c r="C32" s="2">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="D32" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>327</v>
+      </c>
+      <c r="C33" s="2">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+      <c r="D33" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
+        <v>328</v>
+      </c>
+      <c r="C34" s="2">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="D34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F34" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>329</v>
+      </c>
+      <c r="C35" s="2">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="D35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F35" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>330</v>
+      </c>
+      <c r="C36" s="2">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="D36" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>331</v>
+      </c>
+      <c r="C37" s="2">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="D37" t="s">
+        <v>29</v>
+      </c>
+      <c r="F37" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
+        <v>332</v>
+      </c>
+      <c r="C38" s="2">
+        <f t="shared" si="1"/>
+        <v>32</v>
+      </c>
+      <c r="D38" t="s">
+        <v>30</v>
+      </c>
+      <c r="F38" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
+        <v>333</v>
+      </c>
+      <c r="C39" s="2">
+        <f t="shared" si="1"/>
+        <v>33</v>
+      </c>
+      <c r="D39" t="s">
+        <v>31</v>
+      </c>
+      <c r="F39" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="B40" t="s">
+        <v>334</v>
+      </c>
+      <c r="C40" s="2">
+        <f t="shared" si="1"/>
+        <v>34</v>
+      </c>
+      <c r="D40" t="s">
+        <v>32</v>
+      </c>
+      <c r="F40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
+        <v>335</v>
+      </c>
+      <c r="C41" s="2">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="D41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
+        <v>336</v>
+      </c>
+      <c r="C42" s="2">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="D42" t="s">
+        <v>34</v>
+      </c>
+      <c r="F42" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>337</v>
+      </c>
+      <c r="C43" s="2">
+        <f t="shared" si="1"/>
+        <v>37</v>
+      </c>
+      <c r="D43" t="s">
+        <v>35</v>
+      </c>
+      <c r="F43" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>338</v>
+      </c>
+      <c r="C44" s="2">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="D44" t="s">
+        <v>36</v>
+      </c>
+      <c r="F44" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="B45" t="s">
+        <v>339</v>
+      </c>
+      <c r="C45" s="2">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="D45" t="s">
+        <v>37</v>
+      </c>
+      <c r="F45" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="B46" t="s">
+        <v>340</v>
+      </c>
+      <c r="C46" s="2">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="D46" t="s">
+        <v>38</v>
+      </c>
+      <c r="F46" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+      <c r="B47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C47" s="2">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="D47" t="s">
+        <v>39</v>
+      </c>
+      <c r="F47" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="B48" t="s">
+        <v>342</v>
+      </c>
+      <c r="C48" s="2">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+      <c r="D48" t="s">
+        <v>40</v>
+      </c>
+      <c r="F48" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <f t="shared" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="B49" t="s">
+        <v>343</v>
+      </c>
+      <c r="C49" s="2">
+        <f t="shared" si="1"/>
+        <v>43</v>
+      </c>
+      <c r="D49" t="s">
+        <v>41</v>
+      </c>
+      <c r="F49" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>344</v>
+      </c>
+      <c r="C50" s="2">
+        <f t="shared" si="1"/>
+        <v>44</v>
+      </c>
+      <c r="D50" t="s">
+        <v>42</v>
+      </c>
+      <c r="F50" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="B51" t="s">
+        <v>345</v>
+      </c>
+      <c r="C51" s="2">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="D51" t="s">
+        <v>43</v>
+      </c>
+      <c r="F51" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="B52" t="s">
+        <v>346</v>
+      </c>
+      <c r="C52" s="2">
+        <f t="shared" si="1"/>
+        <v>46</v>
+      </c>
+      <c r="D52" t="s">
+        <v>44</v>
+      </c>
+      <c r="F52" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
+      <c r="B53" t="s">
+        <v>347</v>
+      </c>
+      <c r="C53" s="2">
+        <f t="shared" si="1"/>
+        <v>47</v>
+      </c>
+      <c r="D53" t="s">
+        <v>45</v>
+      </c>
+      <c r="F53" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="2">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>348</v>
+      </c>
+      <c r="C54" s="2">
+        <f t="shared" si="1"/>
+        <v>48</v>
+      </c>
+      <c r="D54" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="2">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="B55" t="s">
+        <v>349</v>
+      </c>
+      <c r="C55" s="2">
+        <f t="shared" si="1"/>
+        <v>49</v>
+      </c>
+      <c r="D55" t="s">
+        <v>47</v>
+      </c>
+      <c r="F55" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="B56" t="s">
+        <v>350</v>
+      </c>
+      <c r="C56" s="2">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="D56" t="s">
+        <v>48</v>
+      </c>
+      <c r="F56" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="2">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="B57" t="s">
+        <v>351</v>
+      </c>
+      <c r="C57" s="2">
+        <f t="shared" si="1"/>
+        <v>51</v>
+      </c>
+      <c r="D57" t="s">
+        <v>49</v>
+      </c>
+      <c r="F57" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <f t="shared" si="0"/>
+        <v>56</v>
+      </c>
+      <c r="B58" t="s">
+        <v>352</v>
+      </c>
+      <c r="C58" s="2">
+        <f t="shared" si="1"/>
+        <v>52</v>
+      </c>
+      <c r="D58" t="s">
+        <v>50</v>
+      </c>
+      <c r="F58" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="2">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+      <c r="B59" t="s">
+        <v>353</v>
+      </c>
+      <c r="C59" s="2">
+        <f t="shared" si="1"/>
+        <v>53</v>
+      </c>
+      <c r="D59" t="s">
+        <v>51</v>
+      </c>
+      <c r="F59" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="2">
+        <f t="shared" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>354</v>
+      </c>
+      <c r="C60" s="2">
+        <f t="shared" si="1"/>
+        <v>54</v>
+      </c>
+      <c r="D60" t="s">
+        <v>52</v>
+      </c>
+      <c r="F60" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
+        <f t="shared" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>355</v>
+      </c>
+      <c r="C61" s="2">
+        <f t="shared" si="1"/>
+        <v>55</v>
+      </c>
+      <c r="D61" t="s">
+        <v>53</v>
+      </c>
+      <c r="F61" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="B62" t="s">
+        <v>356</v>
+      </c>
+      <c r="C62" s="2">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+      <c r="D62" t="s">
+        <v>54</v>
+      </c>
+      <c r="F62" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="2">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>357</v>
+      </c>
+      <c r="C63" s="2">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="D63" t="s">
+        <v>55</v>
+      </c>
+      <c r="F63" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="2">
+        <f t="shared" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>358</v>
+      </c>
+      <c r="C64" s="2">
+        <f t="shared" si="1"/>
+        <v>58</v>
+      </c>
+      <c r="D64" t="s">
+        <v>56</v>
+      </c>
+      <c r="F64" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="2">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="B65" t="s">
+        <v>359</v>
+      </c>
+      <c r="C65" s="2">
+        <f t="shared" si="1"/>
+        <v>59</v>
+      </c>
+      <c r="D65" t="s">
+        <v>57</v>
+      </c>
+      <c r="F65" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="2">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>360</v>
+      </c>
+      <c r="C66" s="2">
+        <f t="shared" si="1"/>
+        <v>60</v>
+      </c>
+      <c r="D66" t="s">
+        <v>58</v>
+      </c>
+      <c r="F66" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="2">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>361</v>
+      </c>
+      <c r="C67" s="2">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="D67" t="s">
+        <v>59</v>
+      </c>
+      <c r="F67" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="2">
+        <f t="shared" ref="A68:A95" si="2">A67+1</f>
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>362</v>
+      </c>
+      <c r="C68" s="2">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="D68" t="s">
+        <v>60</v>
+      </c>
+      <c r="F68" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="2">
+        <f t="shared" si="2"/>
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>363</v>
+      </c>
+      <c r="C69" s="2">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="D69" t="s">
+        <v>61</v>
+      </c>
+      <c r="F69" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="2">
+        <f t="shared" si="2"/>
+        <v>68</v>
+      </c>
+      <c r="B70" t="s">
+        <v>364</v>
+      </c>
+      <c r="C70" s="2">
+        <f t="shared" si="1"/>
+        <v>64</v>
+      </c>
+      <c r="D70" t="s">
+        <v>62</v>
+      </c>
+      <c r="F70" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="2">
+        <f t="shared" si="2"/>
+        <v>69</v>
+      </c>
+      <c r="B71" t="s">
+        <v>365</v>
+      </c>
+      <c r="C71" s="2">
+        <f t="shared" si="1"/>
+        <v>65</v>
+      </c>
+      <c r="D71" t="s">
+        <v>63</v>
+      </c>
+      <c r="F71" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="2">
+        <f t="shared" si="2"/>
+        <v>70</v>
+      </c>
+      <c r="B72" t="s">
+        <v>366</v>
+      </c>
+      <c r="C72" s="2">
+        <f t="shared" ref="C72:C87" si="3">+C71+1</f>
+        <v>66</v>
+      </c>
+      <c r="D72" t="s">
+        <v>64</v>
+      </c>
+      <c r="F72" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="2">
+        <f t="shared" si="2"/>
+        <v>71</v>
+      </c>
+      <c r="B73" t="s">
+        <v>367</v>
+      </c>
+      <c r="C73" s="2">
+        <f t="shared" si="3"/>
+        <v>67</v>
+      </c>
+      <c r="D73" t="s">
+        <v>65</v>
+      </c>
+      <c r="F73" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="2">
+        <f t="shared" si="2"/>
+        <v>72</v>
+      </c>
+      <c r="B74" t="s">
+        <v>368</v>
+      </c>
+      <c r="C74" s="2">
+        <f t="shared" si="3"/>
+        <v>68</v>
+      </c>
+      <c r="D74" t="s">
+        <v>66</v>
+      </c>
+      <c r="F74" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="2">
+        <f t="shared" si="2"/>
+        <v>73</v>
+      </c>
+      <c r="B75" t="s">
+        <v>369</v>
+      </c>
+      <c r="C75" s="2">
+        <f t="shared" si="3"/>
+        <v>69</v>
+      </c>
+      <c r="D75" t="s">
+        <v>67</v>
+      </c>
+      <c r="F75" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="2">
+        <f t="shared" si="2"/>
+        <v>74</v>
+      </c>
+      <c r="B76" t="s">
+        <v>370</v>
+      </c>
+      <c r="C76" s="2">
+        <f t="shared" si="3"/>
+        <v>70</v>
+      </c>
+      <c r="D76" t="s">
+        <v>68</v>
+      </c>
+      <c r="F76" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="2">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+      <c r="B77" t="s">
+        <v>371</v>
+      </c>
+      <c r="C77" s="2">
+        <f t="shared" si="3"/>
+        <v>71</v>
+      </c>
+      <c r="D77" t="s">
+        <v>69</v>
+      </c>
+      <c r="F77" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="2">
+        <f t="shared" si="2"/>
+        <v>76</v>
+      </c>
+      <c r="B78" t="s">
+        <v>372</v>
+      </c>
+      <c r="C78" s="2">
+        <f t="shared" si="3"/>
+        <v>72</v>
+      </c>
+      <c r="D78" t="s">
+        <v>70</v>
+      </c>
+      <c r="F78" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="2">
+        <f t="shared" si="2"/>
+        <v>77</v>
+      </c>
+      <c r="B79" t="s">
+        <v>373</v>
+      </c>
+      <c r="C79" s="2">
+        <f t="shared" si="3"/>
+        <v>73</v>
+      </c>
+      <c r="D79" t="s">
+        <v>71</v>
+      </c>
+      <c r="F79" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="2">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
+      <c r="B80" t="s">
+        <v>374</v>
+      </c>
+      <c r="C80" s="2">
+        <f t="shared" si="3"/>
+        <v>74</v>
+      </c>
+      <c r="D80" t="s">
+        <v>72</v>
+      </c>
+      <c r="F80" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="2">
+        <f t="shared" si="2"/>
+        <v>79</v>
+      </c>
+      <c r="B81" t="s">
+        <v>375</v>
+      </c>
+      <c r="C81" s="2">
+        <f t="shared" si="3"/>
+        <v>75</v>
+      </c>
+      <c r="D81" t="s">
+        <v>73</v>
+      </c>
+      <c r="F81" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="2">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="B82" t="s">
+        <v>376</v>
+      </c>
+      <c r="C82" s="2">
+        <f t="shared" si="3"/>
+        <v>76</v>
+      </c>
+      <c r="D82" t="s">
+        <v>74</v>
+      </c>
+      <c r="F82" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="2">
+        <f t="shared" si="2"/>
+        <v>81</v>
+      </c>
+      <c r="B83" t="s">
+        <v>377</v>
+      </c>
+      <c r="C83" s="2">
+        <f t="shared" si="3"/>
+        <v>77</v>
+      </c>
+      <c r="D83" t="s">
+        <v>75</v>
+      </c>
+      <c r="F83" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="2">
+        <f t="shared" si="2"/>
+        <v>82</v>
+      </c>
+      <c r="B84" t="s">
+        <v>378</v>
+      </c>
+      <c r="C84" s="2">
+        <f t="shared" si="3"/>
+        <v>78</v>
+      </c>
+      <c r="D84" t="s">
+        <v>76</v>
+      </c>
+      <c r="F84" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="2">
+        <f t="shared" si="2"/>
+        <v>83</v>
+      </c>
+      <c r="B85" t="s">
+        <v>379</v>
+      </c>
+      <c r="C85" s="2">
+        <f t="shared" si="3"/>
+        <v>79</v>
+      </c>
+      <c r="D85" t="s">
+        <v>77</v>
+      </c>
+      <c r="F85" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="2">
+        <f t="shared" si="2"/>
+        <v>84</v>
+      </c>
+      <c r="B86" t="s">
+        <v>380</v>
+      </c>
+      <c r="C86" s="2">
+        <f t="shared" si="3"/>
+        <v>80</v>
+      </c>
+      <c r="D86" t="s">
+        <v>78</v>
+      </c>
+      <c r="F86" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="2">
+        <f t="shared" si="2"/>
+        <v>85</v>
+      </c>
+      <c r="B87" t="s">
+        <v>381</v>
+      </c>
+      <c r="C87" s="2">
+        <f t="shared" si="3"/>
+        <v>81</v>
+      </c>
+      <c r="D87" t="s">
+        <v>79</v>
+      </c>
+      <c r="F87" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="2">
+        <f t="shared" si="2"/>
+        <v>86</v>
+      </c>
+      <c r="B88" t="s">
+        <v>382</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E88" t="s">
+        <v>189</v>
+      </c>
+      <c r="F88" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="2">
+        <f t="shared" si="2"/>
+        <v>87</v>
+      </c>
+      <c r="B89" t="s">
+        <v>383</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E89" t="s">
+        <v>191</v>
+      </c>
+      <c r="F89" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <f t="shared" si="2"/>
+        <v>88</v>
+      </c>
+      <c r="B90" t="s">
+        <v>384</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E90" t="s">
+        <v>187</v>
+      </c>
+      <c r="F90" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" s="2">
+        <f t="shared" si="2"/>
+        <v>89</v>
+      </c>
+      <c r="B91" t="s">
+        <v>385</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E91" t="s">
+        <v>190</v>
+      </c>
+      <c r="F91" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="2">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="B92" t="s">
+        <v>386</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E92" t="s">
+        <v>189</v>
+      </c>
+      <c r="F92" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="2">
+        <f t="shared" si="2"/>
+        <v>91</v>
+      </c>
+      <c r="B93" t="s">
+        <v>387</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E93" t="s">
+        <v>191</v>
+      </c>
+      <c r="F93" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="2">
+        <f t="shared" si="2"/>
+        <v>92</v>
+      </c>
+      <c r="B94" t="s">
+        <v>388</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E94" t="s">
+        <v>187</v>
+      </c>
       <c r="F94" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="2">
+        <f t="shared" si="2"/>
+        <v>93</v>
+      </c>
+      <c r="B95" t="s">
+        <v>389</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E95" t="s">
+        <v>190</v>
+      </c>
+      <c r="F95" t="s">
         <v>194</v>
       </c>
     </row>

</xml_diff>